<commit_message>
long time no C - ommit
</commit_message>
<xml_diff>
--- a/R/data/generated/tables/compilation_basic_top_200.xlsx
+++ b/R/data/generated/tables/compilation_basic_top_200.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maxshore/Documents/Unibe/MasterThesis/masterthesis/R/data/generated/tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFC95357-E278-DB43-A356-C5E1584789CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43832233-5A2C-BA43-87B9-EF4414401F88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1180" yWindow="1500" windowWidth="27240" windowHeight="15940" xr2:uid="{CDDC8DA5-CD77-1148-A3F8-1C791DE9C1CD}"/>
   </bookViews>
@@ -160,7 +160,35 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="medium">
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
         <color indexed="64"/>
       </top>
       <bottom style="medium">
@@ -169,186 +197,137 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom style="medium">
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="medium">
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom style="medium">
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="medium">
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
         <color indexed="64"/>
       </right>
-      <top/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
+      <left style="thin">
         <color indexed="64"/>
       </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
+      <right style="thin">
         <color indexed="64"/>
       </right>
       <top style="medium">
         <color indexed="64"/>
       </top>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="11" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="11" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="11" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -684,12 +663,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D057A2C3-010F-094C-AF50-E5EA3FC35C48}">
-  <dimension ref="F13:V22"/>
+  <dimension ref="F13:S19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="16" max="16" width="9.5" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="13" spans="6:22" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="6:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="F14" s="1"/>
+    <row r="13" spans="6:19" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="6:19" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="F14" s="3"/>
       <c r="G14" s="2" t="s">
         <v>0</v>
       </c>
@@ -720,364 +702,237 @@
       <c r="P14" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="Q14" s="3" t="s">
+      <c r="Q14" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="R14" s="4"/>
+      <c r="R14" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="S14" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="T14" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="U14" s="4"/>
-      <c r="V14" s="2"/>
     </row>
-    <row r="15" spans="6:22" x14ac:dyDescent="0.2">
-      <c r="F15" s="5" t="s">
+    <row r="15" spans="6:19" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="F15" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G15" s="6">
+      <c r="G15" s="17">
         <v>0.52997187000000001</v>
       </c>
-      <c r="H15" s="6">
+      <c r="H15" s="12">
         <v>6.8807499999999997E-3</v>
       </c>
-      <c r="I15" s="6">
+      <c r="I15" s="12">
         <v>1.71748E-3</v>
       </c>
-      <c r="J15" s="6">
+      <c r="J15" s="12">
         <v>0.16152073</v>
       </c>
-      <c r="K15" s="6">
+      <c r="K15" s="12">
         <v>2.9140799999999999E-3</v>
       </c>
-      <c r="L15" s="6">
+      <c r="L15" s="12">
         <v>2.1450810000000001E-2</v>
       </c>
-      <c r="M15" s="6">
+      <c r="M15" s="12">
         <v>0.20684541000000001</v>
       </c>
-      <c r="N15" s="6">
+      <c r="N15" s="12">
         <v>5.4320899999999997E-3</v>
       </c>
-      <c r="O15" s="6">
+      <c r="O15" s="12">
         <v>3.3302499999999999E-3</v>
       </c>
-      <c r="P15" s="6">
+      <c r="P15" s="12">
         <v>5.2266609999999998E-2</v>
       </c>
-      <c r="Q15" s="23">
+      <c r="Q15" s="16">
         <v>1.38949E-3</v>
       </c>
-      <c r="R15" s="24"/>
-      <c r="S15" s="25">
+      <c r="R15" s="10">
         <v>4.727E-4</v>
       </c>
-      <c r="T15" s="23">
+      <c r="S15" s="10">
         <v>5.8077500000000004E-3</v>
       </c>
-      <c r="U15" s="24"/>
-      <c r="V15" s="5"/>
     </row>
-    <row r="16" spans="6:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="F16" s="8"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="9"/>
-      <c r="I16" s="9"/>
-      <c r="J16" s="9"/>
-      <c r="K16" s="9"/>
-      <c r="L16" s="9"/>
-      <c r="M16" s="9"/>
-      <c r="N16" s="9"/>
-      <c r="O16" s="9"/>
-      <c r="P16" s="9"/>
-      <c r="Q16" s="26"/>
-      <c r="R16" s="27"/>
-      <c r="S16" s="28"/>
-      <c r="T16" s="26"/>
-      <c r="U16" s="27"/>
-      <c r="V16" s="8"/>
+    <row r="16" spans="6:19" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="F16" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G16" s="4">
+        <v>3.9381619999999999E-2</v>
+      </c>
+      <c r="H16" s="11">
+        <v>1.01461E-3</v>
+      </c>
+      <c r="I16" s="5">
+        <v>5.2934E-4</v>
+      </c>
+      <c r="J16" s="5">
+        <v>1.398367E-2</v>
+      </c>
+      <c r="K16" s="5">
+        <v>3.2841000000000001E-4</v>
+      </c>
+      <c r="L16" s="5">
+        <v>2.2719099999999998E-3</v>
+      </c>
+      <c r="M16" s="5">
+        <v>1.99188E-2</v>
+      </c>
+      <c r="N16" s="5">
+        <v>7.3532000000000003E-4</v>
+      </c>
+      <c r="O16" s="5">
+        <v>4.8329999999999998E-4</v>
+      </c>
+      <c r="P16" s="5">
+        <v>5.3669800000000004E-3</v>
+      </c>
+      <c r="Q16" s="11">
+        <v>2.4835999999999999E-4</v>
+      </c>
+      <c r="R16" s="13">
+        <v>6.7899999999999997E-5</v>
+      </c>
+      <c r="S16" s="5">
+        <v>4.0999999999999999E-4</v>
+      </c>
     </row>
-    <row r="17" spans="6:22" x14ac:dyDescent="0.2">
-      <c r="F17" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="G17" s="6">
-        <v>3.9381619999999999E-2</v>
+    <row r="17" spans="6:19" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="F17" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G17" s="14">
+        <v>0.54038850000000005</v>
       </c>
       <c r="H17" s="6">
-        <v>1.01461E-3</v>
+        <v>6.65534E-3</v>
       </c>
       <c r="I17" s="6">
-        <v>5.2934E-4</v>
+        <v>1.87463E-3</v>
       </c>
       <c r="J17" s="6">
-        <v>1.398367E-2</v>
-      </c>
-      <c r="K17" s="6">
-        <v>3.2841000000000001E-4</v>
-      </c>
-      <c r="L17" s="6">
-        <v>2.2719099999999998E-3</v>
+        <v>0.15847067000000001</v>
+      </c>
+      <c r="K17" s="15">
+        <v>2.8380599999999999E-3</v>
+      </c>
+      <c r="L17" s="5">
+        <v>2.084043E-2</v>
       </c>
       <c r="M17" s="6">
-        <v>1.99188E-2</v>
+        <v>0.20279606999999999</v>
       </c>
       <c r="N17" s="6">
-        <v>7.3532000000000003E-4</v>
+        <v>5.3393099999999999E-3</v>
       </c>
       <c r="O17" s="6">
-        <v>4.8329999999999998E-4</v>
+        <v>3.2376000000000002E-3</v>
       </c>
       <c r="P17" s="6">
-        <v>5.3669800000000004E-3</v>
-      </c>
-      <c r="Q17" s="11">
-        <v>2.4835999999999999E-4</v>
-      </c>
-      <c r="R17" s="12"/>
-      <c r="S17" s="13">
-        <v>6.7899999999999997E-5</v>
-      </c>
-      <c r="T17" s="11">
-        <v>4.0999999999999999E-4</v>
-      </c>
-      <c r="U17" s="12"/>
-      <c r="V17" s="5"/>
+        <v>5.000599E-2</v>
+      </c>
+      <c r="Q17" s="15">
+        <v>1.3458000000000001E-3</v>
+      </c>
+      <c r="R17" s="6">
+        <v>4.7259999999999999E-4</v>
+      </c>
+      <c r="S17" s="6">
+        <v>5.7349999999999996E-3</v>
+      </c>
     </row>
-    <row r="18" spans="6:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="F18" s="8"/>
-      <c r="G18" s="9"/>
-      <c r="H18" s="9"/>
-      <c r="I18" s="9"/>
-      <c r="J18" s="9"/>
-      <c r="K18" s="9"/>
-      <c r="L18" s="9"/>
-      <c r="M18" s="9"/>
-      <c r="N18" s="9"/>
-      <c r="O18" s="9"/>
-      <c r="P18" s="9"/>
-      <c r="Q18" s="14"/>
-      <c r="R18" s="15"/>
-      <c r="S18" s="10"/>
-      <c r="T18" s="14"/>
-      <c r="U18" s="15"/>
-      <c r="V18" s="8"/>
+    <row r="18" spans="6:19" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="F18" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G18" s="4">
+        <v>0.52639921999999995</v>
+      </c>
+      <c r="H18" s="5">
+        <v>6.9580600000000003E-3</v>
+      </c>
+      <c r="I18" s="6">
+        <v>1.66358E-3</v>
+      </c>
+      <c r="J18" s="5">
+        <v>0.16256682</v>
+      </c>
+      <c r="K18" s="5">
+        <v>2.9401599999999998E-3</v>
+      </c>
+      <c r="L18" s="6">
+        <v>2.1660160000000001E-2</v>
+      </c>
+      <c r="M18" s="5">
+        <v>0.20823422999999999</v>
+      </c>
+      <c r="N18" s="5">
+        <v>5.4638999999999998E-3</v>
+      </c>
+      <c r="O18" s="5">
+        <v>3.3620199999999999E-3</v>
+      </c>
+      <c r="P18" s="5">
+        <v>5.3041949999999997E-2</v>
+      </c>
+      <c r="Q18" s="5">
+        <v>1.4044699999999999E-3</v>
+      </c>
+      <c r="R18" s="5">
+        <v>4.7272999999999998E-4</v>
+      </c>
+      <c r="S18" s="5">
+        <v>5.8326999999999997E-3</v>
+      </c>
     </row>
-    <row r="19" spans="6:22" x14ac:dyDescent="0.2">
-      <c r="F19" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G19" s="25">
-        <v>0.54038850000000005</v>
-      </c>
-      <c r="H19" s="25">
-        <v>6.65534E-3</v>
-      </c>
-      <c r="I19" s="25">
-        <v>1.87463E-3</v>
-      </c>
-      <c r="J19" s="25">
-        <v>0.15847067000000001</v>
-      </c>
-      <c r="K19" s="25">
-        <v>2.8380599999999999E-3</v>
-      </c>
-      <c r="L19" s="6">
-        <v>2.084043E-2</v>
-      </c>
-      <c r="M19" s="25">
-        <v>0.20279606999999999</v>
-      </c>
-      <c r="N19" s="25">
-        <v>5.3393099999999999E-3</v>
-      </c>
-      <c r="O19" s="25">
-        <v>3.2376000000000002E-3</v>
-      </c>
-      <c r="P19" s="25">
-        <v>5.000599E-2</v>
-      </c>
-      <c r="Q19" s="23">
-        <v>1.3458000000000001E-3</v>
-      </c>
-      <c r="R19" s="24"/>
-      <c r="S19" s="25">
-        <v>4.7259999999999999E-4</v>
-      </c>
-      <c r="T19" s="23">
-        <v>5.7349999999999996E-3</v>
-      </c>
-      <c r="U19" s="24"/>
-      <c r="V19" s="5"/>
-    </row>
-    <row r="20" spans="6:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="F20" s="8"/>
-      <c r="G20" s="28"/>
-      <c r="H20" s="28"/>
-      <c r="I20" s="28"/>
-      <c r="J20" s="28"/>
-      <c r="K20" s="28"/>
-      <c r="L20" s="9"/>
-      <c r="M20" s="28"/>
-      <c r="N20" s="28"/>
-      <c r="O20" s="28"/>
-      <c r="P20" s="28"/>
-      <c r="Q20" s="26"/>
-      <c r="R20" s="27"/>
-      <c r="S20" s="28"/>
-      <c r="T20" s="26"/>
-      <c r="U20" s="27"/>
-      <c r="V20" s="8"/>
-    </row>
-    <row r="21" spans="6:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="F21" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="G21" s="17">
-        <v>0.52639921999999995</v>
-      </c>
-      <c r="H21" s="17">
-        <v>6.9580600000000003E-3</v>
-      </c>
-      <c r="I21" s="7">
-        <v>1.66358E-3</v>
-      </c>
-      <c r="J21" s="17">
-        <v>0.16256682</v>
-      </c>
-      <c r="K21" s="17">
-        <v>2.9401599999999998E-3</v>
-      </c>
-      <c r="L21" s="7">
-        <v>2.1660160000000001E-2</v>
-      </c>
-      <c r="M21" s="17">
-        <v>0.20823422999999999</v>
-      </c>
-      <c r="N21" s="17">
-        <v>5.4638999999999998E-3</v>
-      </c>
-      <c r="O21" s="17">
-        <v>3.3620199999999999E-3</v>
-      </c>
-      <c r="P21" s="17">
-        <v>5.3041949999999997E-2</v>
-      </c>
-      <c r="Q21" s="18">
-        <v>1.4044699999999999E-3</v>
-      </c>
-      <c r="R21" s="19"/>
-      <c r="S21" s="17">
-        <v>4.7272999999999998E-4</v>
-      </c>
-      <c r="T21" s="18">
-        <v>5.8326999999999997E-3</v>
-      </c>
-      <c r="U21" s="19"/>
-      <c r="V21" s="20"/>
-    </row>
-    <row r="22" spans="6:22" ht="29" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="F22" s="16" t="s">
+    <row r="19" spans="6:19" ht="29" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="F19" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="G22" s="21">
+      <c r="G19" s="7">
         <v>2.926148E-15</v>
       </c>
-      <c r="H22" s="21">
+      <c r="H19" s="8">
         <v>4.3044579999999998E-8</v>
       </c>
-      <c r="I22" s="21">
+      <c r="I19" s="8">
         <v>7.5178460000000004E-15</v>
       </c>
-      <c r="J22" s="21">
+      <c r="J19" s="8">
         <v>1.06106E-11</v>
       </c>
-      <c r="K22" s="21">
+      <c r="K19" s="8">
         <v>2.1883179999999999E-9</v>
       </c>
-      <c r="L22" s="21">
+      <c r="L19" s="8">
         <v>6.791419E-12</v>
       </c>
-      <c r="M22" s="21">
+      <c r="M19" s="8">
         <v>9.2872549999999993E-9</v>
       </c>
-      <c r="N22" s="21">
+      <c r="N19" s="8">
         <v>6.0589610000000001E-5</v>
       </c>
-      <c r="O22" s="21">
+      <c r="O19" s="8">
         <v>9.8061649999999991E-7</v>
       </c>
-      <c r="P22" s="20" t="s">
+      <c r="P19" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="Q22" s="22">
+      <c r="Q19" s="8">
         <v>3.4699999999999998E-4</v>
       </c>
-      <c r="R22" s="4"/>
-      <c r="S22" s="20" t="s">
+      <c r="R19" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="T22" s="3" t="s">
+      <c r="S19" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="U22" s="4"/>
-      <c r="V22" s="20"/>
     </row>
   </sheetData>
-  <mergeCells count="50">
-    <mergeCell ref="T19:U20"/>
-    <mergeCell ref="Q15:R16"/>
-    <mergeCell ref="S15:S16"/>
-    <mergeCell ref="T15:U16"/>
-    <mergeCell ref="Q22:R22"/>
-    <mergeCell ref="T22:U22"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="H19:H20"/>
-    <mergeCell ref="I19:I20"/>
-    <mergeCell ref="J19:J20"/>
-    <mergeCell ref="K19:K20"/>
-    <mergeCell ref="M19:M20"/>
-    <mergeCell ref="N19:N20"/>
-    <mergeCell ref="O19:O20"/>
-    <mergeCell ref="T17:U18"/>
-    <mergeCell ref="V17:V18"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="L19:L20"/>
-    <mergeCell ref="V19:V20"/>
-    <mergeCell ref="Q21:R21"/>
-    <mergeCell ref="T21:U21"/>
-    <mergeCell ref="P19:P20"/>
-    <mergeCell ref="Q19:R20"/>
-    <mergeCell ref="S19:S20"/>
-    <mergeCell ref="L17:L18"/>
-    <mergeCell ref="M17:M18"/>
-    <mergeCell ref="N17:N18"/>
-    <mergeCell ref="O17:O18"/>
-    <mergeCell ref="P17:P18"/>
-    <mergeCell ref="Q17:R18"/>
-    <mergeCell ref="N15:N16"/>
-    <mergeCell ref="O15:O16"/>
-    <mergeCell ref="P15:P16"/>
-    <mergeCell ref="V15:V16"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="G17:G18"/>
-    <mergeCell ref="H17:H18"/>
-    <mergeCell ref="I17:I18"/>
-    <mergeCell ref="J17:J18"/>
-    <mergeCell ref="K17:K18"/>
-    <mergeCell ref="Q14:R14"/>
-    <mergeCell ref="T14:U14"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="G15:G16"/>
-    <mergeCell ref="H15:H16"/>
-    <mergeCell ref="I15:I16"/>
-    <mergeCell ref="J15:J16"/>
-    <mergeCell ref="K15:K16"/>
-    <mergeCell ref="L15:L16"/>
-    <mergeCell ref="M15:M16"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>